<commit_message>
commiited on 16 feb
</commit_message>
<xml_diff>
--- a/testData/demowebshop.xlsx
+++ b/testData/demowebshop.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="loginFunctions" sheetId="1" r:id="rId1"/>
     <sheet name="socialMediaFunctions" sheetId="3" r:id="rId2"/>
-    <sheet name="RegisterPageFunctions" sheetId="2" r:id="rId3"/>
+    <sheet name="registerPageActions" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>password</t>
   </si>
@@ -49,12 +49,6 @@
     <t>confirmPassword</t>
   </si>
   <si>
-    <t>santhoshkumarm</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
     <t>priy.sa@med.com</t>
   </si>
   <si>
@@ -62,6 +56,30 @@
   </si>
   <si>
     <t>https://www.facebook.com/nopCommerce</t>
+  </si>
+  <si>
+    <t>joseph</t>
+  </si>
+  <si>
+    <t>murphy</t>
+  </si>
+  <si>
+    <t>Saibaba1@4</t>
+  </si>
+  <si>
+    <t>Saibaba1@5</t>
+  </si>
+  <si>
+    <t>akash</t>
+  </si>
+  <si>
+    <t>m12</t>
+  </si>
+  <si>
+    <t>kuga@g.com</t>
+  </si>
+  <si>
+    <t>kuga1@g.con</t>
   </si>
 </sst>
 </file>
@@ -407,7 +425,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -440,12 +458,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -456,10 +474,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="18.140625" customWidth="1"/>
@@ -484,27 +502,46 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>2</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1"/>
-    <hyperlink ref="D2" r:id="rId2"/>
-    <hyperlink ref="E2" r:id="rId3"/>
+    <hyperlink ref="E2:E3" r:id="rId1" display="Saibaba1@3"/>
+    <hyperlink ref="D2:D3" r:id="rId2" display="Saibaba1@3"/>
+    <hyperlink ref="C2" r:id="rId3"/>
+    <hyperlink ref="C3" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>